<commit_message>
0.8.1 Document HTTP status codes, and documentation
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-retina-ai-gradability-cs.xlsx
+++ b/docs/CodeSystem-retina-ai-gradability-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.8.0</t>
+    <t>0.8.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-17</t>
+    <t>2026-04-28</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -147,7 +147,7 @@
     <t>Good</t>
   </si>
   <si>
-    <t>The data quality is sufficient for it to be processed by an AI grading algorithm.</t>
+    <t>The submitted set of images is sufficient for evaluation.</t>
   </si>
   <si>
     <t>not-gradable</t>
@@ -156,7 +156,7 @@
     <t>Not gradable</t>
   </si>
   <si>
-    <t>The data quality is insufficient for it to be processed by an AI grading algorithm.</t>
+    <t>The submitted set of images is insufficient for evaluation.</t>
   </si>
 </sst>
 </file>

</xml_diff>